<commit_message>
Added a universal checker to idenitfy required courses that are not offered at one's home college (namely CSE 12 requirement for Comp Eng out of EVC) updated worksheet.xlsx to have comsc 077 for UCSD comp eng
</commit_message>
<xml_diff>
--- a/worksheet.xlsx
+++ b/worksheet.xlsx
@@ -519,7 +519,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A37"/>
+  <dimension ref="A1:A43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -739,26 +739,64 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>KNOWN LIMITATION: convert_worksheet.py currently reads 'Elective Groups'/'Elective Options'</t>
+          <t>AUTOMATIC CROSS-CCC GAP CHECK: every time you run build_dist.py, it automatically checks every</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>for your own reference but does NOT yet feed pick-N-of-M logic into the app -- the app's</t>
+          <t>required-but-unarticulated course at every CCC against every OTHER CCC's catalog -- if another</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>data model only understands flat 'required' lists right now. The data is captured here so</t>
+          <t>CCC in your dataset offers it, it's reported on the console and written to</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>dist/cross_ccc_alternatives.json. This runs on every future addition too, not just today's data --</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>no need to check for this by hand.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>KNOWN LIMITATION: convert_worksheet.py currently reads 'Elective Groups'/'Elective Options'</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>for your own reference but does NOT yet feed pick-N-of-M logic into the app -- the app's</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>data model only understands flat 'required' lists right now. The data is captured here so</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
         <is>
           <t>it isn't lost, ready for whenever the app/frontend is extended to actually display choices.</t>
         </is>
@@ -955,7 +993,7 @@
       </c>
       <c r="E2" s="7" t="inlineStr">
         <is>
-          <t>CONFIRMED via actual UCSD ASSIST agreements (both De Anza and EVC PDFs agree). Official 'General Advice' list: MATH 20A/20B/20C (calc1/2/3), MATH 20D (diffeq), MATH 18 (linalg), calc-based physics series (physics1/2/3), CSE 8B-or-11 (prog1), CSE 12 (prog2), CSE 20 (discrete). CORRECTION from an earlier version of this sheet: discrete math IS explicitly required (previously left unmarked); Computer Organization is NOT in the official required list (previously marked required in error) -- it appears in the detailed per-CCC table but not the summary bullet list, so treat it as unconfirmed.</t>
+          <t>CONFIRMED via actual UCSD ASSIST agreements (both De Anza and EVC PDFs agree). Official 'General Advice' list: MATH 20A/20B/20C (calc1/2/3), MATH 20D (diffeq), MATH 18 (linalg), calc-based physics series (physics1/2/3), CSE 8B-or-11 (prog1), CSE 12 (prog2), CSE 20 (discrete). CSE 30 (comporg) is ALSO required -- user confirmed via the live page after this sheet initially left it out because it wasn't in the summary bullet list (only in the detailed per-CCC table). Lesson: the detailed table is the authoritative source; the prose summary isn't necessarily exhaustive.</t>
         </is>
       </c>
       <c r="F2" s="8" t="inlineStr">
@@ -998,7 +1036,11 @@
           <t>X</t>
         </is>
       </c>
-      <c r="N2" s="9" t="n"/>
+      <c r="N2" s="8" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="O2" s="9" t="n"/>
       <c r="P2" s="8" t="inlineStr">
         <is>
@@ -1023,7 +1065,7 @@
       <c r="X2" s="9" t="n"/>
       <c r="Y2" s="10" t="inlineStr">
         <is>
-          <t>Fully confirmed row -- see source note. Computer Organization intentionally left blank (not in official required list).</t>
+          <t>Fully confirmed row, including comporg (CSE 30) -- confirmed against the live page after this sheet initially missed it.</t>
         </is>
       </c>
     </row>
@@ -1242,7 +1284,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="H3 H5 I5 J3 J5 K3 K4 K5 L3 L5 M3 M4 M5 N2 N3 N4 N5 O2 O3 O4 O5 P3 P5 Q3 Q5 R3 R5 S2 S3 S5 T2 T3 T4 T5 U2 U3 U4 U5 V2 V3 V4 W2 W3 W4 W5 X2 X4 X5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H3 H5 I5 J3 J5 K3 K4 K5 L3 L5 M3 M4 M5 N3 N4 N5 O2 O3 O4 O5 P3 P5 Q3 Q5 R3 R5 S2 S3 S5 T2 T3 T4 T5 U2 U3 U4 U5 V2 V3 V4 W2 W3 W4 W5 X2 X4 X5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"X,"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1473,12 +1515,12 @@
       </c>
       <c r="D8" s="8" t="inlineStr">
         <is>
-          <t>COMSC 075 (or CIT 044 Java)</t>
+          <t>CIT 044 (or COMSC 076) for UCSD; CIT 044 (or COMSC 075) for UCI -- differs by receiving school, see limitation note</t>
         </is>
       </c>
       <c r="E8" s="12" t="inlineStr">
         <is>
-          <t>CONFIRMED via actual ASSIST agreement PDFs (2025-2026, this session).</t>
+          <t>SEE LIMITATION NOTE: EVC's prog1 course also differs by receiving school (COMSC 076 for UCSD, COMSC 075 for UCI, both alongside CIT 044) -- same one-cell-per-slot limitation as calc3.</t>
         </is>
       </c>
     </row>
@@ -1498,14 +1540,10 @@
           <t>CIS 22C (or 22CH)</t>
         </is>
       </c>
-      <c r="D9" s="8" t="inlineStr">
-        <is>
-          <t>COMSC 076</t>
-        </is>
-      </c>
+      <c r="D9" s="9" t="n"/>
       <c r="E9" s="12" t="inlineStr">
         <is>
-          <t>CONFIRMED via actual ASSIST agreement PDFs (2025-2026, this session).</t>
+          <t>GAP AT EVC for UCSD Computer Engineering: CSE 12 has no EVC equivalent (confirmed against the live ASSIST page). Students can instead complete it via De Anza College's CIS 22C (or 22CH) -- confirmed on De Anza's own agreement -- by cross-enrolling or taking it there before transfer. This is exactly the kind of gap dist/cross_ccc_alternatives.json now finds automatically on every build.</t>
         </is>
       </c>
     </row>
@@ -1520,9 +1558,21 @@
           <t>Computer Organization</t>
         </is>
       </c>
-      <c r="C10" s="9" t="n"/>
-      <c r="D10" s="9" t="n"/>
-      <c r="E10" s="12" t="n"/>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>CIS 21JA + CIS 21JB + CIS 26B (or CIS 26BH honors) -- inferred by structural parallel with EVC's same 'Complete A or B' section; not read as clearly as EVC's mapping was</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>COMSC 077 (Introduction to Computer Systems)</t>
+        </is>
+      </c>
+      <c r="E10" s="12" t="inlineStr">
+        <is>
+          <t>CONFIRMED via actual ASSIST agreement PDFs (2025-2026, this session).</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1700,9 +1750,21 @@
           <t>Introduction to Psychology</t>
         </is>
       </c>
-      <c r="C18" s="9" t="n"/>
-      <c r="D18" s="9" t="n"/>
-      <c r="E18" s="12" t="n"/>
+      <c r="C18" s="8" t="inlineStr">
+        <is>
+          <t>PSYC C1000 + PSYC 24 for COGS 9A; PSYC C1000 + (PSYC 4 or PSYC 8) for COGS 9C -- differs by which COGS course it satisfies, same limitation pattern as calc3</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>PSYC C1000 + PSYCH 030 for COGS 9A; PSYC C1000 + PSYCH 099 for COGS 9C -- differs by which COGS course it satisfies, same limitation pattern as calc3</t>
+        </is>
+      </c>
+      <c r="E18" s="12" t="inlineStr">
+        <is>
+          <t>SEE LIMITATION NOTE: this slot needs a different course combo depending on whether it's satisfying UCI's COGS 9A or COGS 9C -- same one-cell-per-slot limitation as calc3 and prog1.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Fixed backend to correctly process AP score results
</commit_message>
<xml_diff>
--- a/worksheet.xlsx
+++ b/worksheet.xlsx
@@ -12,7 +12,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CCC Catalog" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Elective Groups" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Elective Options" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slot Reference" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AP Credit" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slot Reference" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -519,7 +520,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A43"/>
+  <dimension ref="A1:A48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -777,26 +778,57 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>KNOWN LIMITATION: convert_worksheet.py currently reads 'Elective Groups'/'Elective Options'</t>
+          <t>AP CREDIT: the 'AP Credit' tab lists which AP exam + minimum score satisfies which slot, sourced</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>for your own reference but does NOT yet feed pick-N-of-M logic into the app -- the app's</t>
+          <t>from official UC AP credit charts (not guessed). build_dist.py turns this into dist/ap_credit.json,</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>data model only understands flat 'required' lists right now. The data is captured here so</t>
+          <t>which the frontend can check against a student's uploaded scores. Add more rows here (AP CS A,</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>AP Physics C, etc.) the same way -- one row per (school, exam, min score, slot).</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>KNOWN LIMITATION: convert_worksheet.py currently reads 'Elective Groups'/'Elective Options'</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>for your own reference but does NOT yet feed pick-N-of-M logic into the app -- the app's</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>data model only understands flat 'required' lists right now. The data is captured here so</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
         <is>
           <t>it isn't lost, ready for whenever the app/frontend is extended to actually display choices.</t>
         </is>
@@ -2003,7 +2035,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D35"/>
+  <dimension ref="A1:D37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -2152,12 +2184,12 @@
       </c>
       <c r="B7" s="13" t="inlineStr">
         <is>
-          <t>physics_2course</t>
+          <t>physics_calc_based</t>
         </is>
       </c>
       <c r="C7" s="14" t="inlineStr">
         <is>
-          <t>EVC PHYS 007A + PHYS 007B (only 2 courses -- EVC has no 3rd physics course option here)</t>
+          <t>EVC PHYS 007A + PHYS 007B (only 2 courses -- EVC has no 3rd course here). This satisfies UCI's CALCULUS-BASED 'Classical Physics' sequence (PHYSICS 7C/7D/7E) specifically.</t>
         </is>
       </c>
       <c r="D7" s="13" t="inlineStr">
@@ -2174,12 +2206,12 @@
       </c>
       <c r="B8" s="13" t="inlineStr">
         <is>
-          <t>physics_2course</t>
+          <t>physics_calc_based</t>
         </is>
       </c>
       <c r="C8" s="14" t="inlineStr">
         <is>
-          <t>EVC PHYS 007A + PHYS 007B (only 2 courses -- EVC has no 3rd physics course option here)</t>
+          <t>EVC PHYS 007A + PHYS 007B (only 2 courses -- EVC has no 3rd course here). This satisfies UCI's CALCULUS-BASED 'Classical Physics' sequence (PHYSICS 7C/7D/7E) specifically.</t>
         </is>
       </c>
       <c r="D8" s="13" t="inlineStr">
@@ -2196,19 +2228,15 @@
       </c>
       <c r="B9" s="13" t="inlineStr">
         <is>
-          <t>statistics</t>
+          <t>physics_algebra_based</t>
         </is>
       </c>
       <c r="C9" s="14" t="inlineStr">
         <is>
-          <t>EVC STAT C1000 (or BUS 060)</t>
-        </is>
-      </c>
-      <c r="D9" s="13" t="inlineStr">
-        <is>
-          <t>stats_gen</t>
-        </is>
-      </c>
+          <t>UCI ALSO separately accepts an ALGEBRA-based 'Basic Physics' sequence (PHYSICS 3A/3B/3C) as an alternative option -- this is NOT the same course sequence as physics1/2/3 above and is NOT interchangeable with it (confirmed: user verified these are non-equivalent). No EVC course has been confirmed against this specific algebra-based track -- do not assume the calc-based mapping above covers it.</t>
+        </is>
+      </c>
+      <c r="D9" s="13" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="13" t="inlineStr">
@@ -2218,15 +2246,19 @@
       </c>
       <c r="B10" s="13" t="inlineStr">
         <is>
-          <t>logic</t>
+          <t>statistics</t>
         </is>
       </c>
       <c r="C10" s="14" t="inlineStr">
         <is>
-          <t>EVC PHIL 090 (Introduction to Logic) -- no matching slot tracked here</t>
-        </is>
-      </c>
-      <c r="D10" s="13" t="inlineStr"/>
+          <t>EVC STAT C1000 (or BUS 060)</t>
+        </is>
+      </c>
+      <c r="D10" s="13" t="inlineStr">
+        <is>
+          <t>stats_gen</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="13" t="inlineStr">
@@ -2236,12 +2268,12 @@
       </c>
       <c r="B11" s="13" t="inlineStr">
         <is>
-          <t>linguistics</t>
+          <t>logic</t>
         </is>
       </c>
       <c r="C11" s="14" t="inlineStr">
         <is>
-          <t>No EVC equivalent exists for any linguistics option (LSCI 3/10/20/51)</t>
+          <t>EVC PHIL 090 (Introduction to Logic) -- no matching slot tracked here</t>
         </is>
       </c>
       <c r="D11" s="13" t="inlineStr"/>
@@ -2254,12 +2286,12 @@
       </c>
       <c r="B12" s="13" t="inlineStr">
         <is>
-          <t>neuro_electives</t>
+          <t>linguistics</t>
         </is>
       </c>
       <c r="C12" s="14" t="inlineStr">
         <is>
-          <t>No EVC equivalent exists for extra neuro electives (BIO SCI 36/37/38)</t>
+          <t>No EVC equivalent exists for any linguistics option (LSCI 3/10/20/51)</t>
         </is>
       </c>
       <c r="D12" s="13" t="inlineStr"/>
@@ -2267,24 +2299,20 @@
     <row r="13">
       <c r="A13" s="13" t="inlineStr">
         <is>
-          <t>uci_cogsci_electives_deanza</t>
+          <t>uci_cogsci_electives_evc</t>
         </is>
       </c>
       <c r="B13" s="13" t="inlineStr">
         <is>
-          <t>programming</t>
+          <t>neuro_electives</t>
         </is>
       </c>
       <c r="C13" s="14" t="inlineStr">
         <is>
-          <t>Programming series: De Anza CIS 40 + CIS 41A + CIS 41B (3 courses)</t>
-        </is>
-      </c>
-      <c r="D13" s="13" t="inlineStr">
-        <is>
-          <t>prog1</t>
-        </is>
-      </c>
+          <t>No EVC equivalent exists for extra neuro electives (BIO SCI 36/37/38)</t>
+        </is>
+      </c>
+      <c r="D13" s="13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="13" t="inlineStr">
@@ -2304,7 +2332,7 @@
       </c>
       <c r="D14" s="13" t="inlineStr">
         <is>
-          <t>prog2</t>
+          <t>prog1</t>
         </is>
       </c>
     </row>
@@ -2316,15 +2344,19 @@
       </c>
       <c r="B15" s="13" t="inlineStr">
         <is>
-          <t>linguistics</t>
+          <t>programming</t>
         </is>
       </c>
       <c r="C15" s="14" t="inlineStr">
         <is>
-          <t>De Anza LING 1 (Introduction to Linguistics) -- real equivalent, unlike EVC</t>
-        </is>
-      </c>
-      <c r="D15" s="13" t="inlineStr"/>
+          <t>Programming series: De Anza CIS 40 + CIS 41A + CIS 41B (3 courses)</t>
+        </is>
+      </c>
+      <c r="D15" s="13" t="inlineStr">
+        <is>
+          <t>prog2</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="13" t="inlineStr">
@@ -2334,12 +2366,12 @@
       </c>
       <c r="B16" s="13" t="inlineStr">
         <is>
-          <t>logic</t>
+          <t>linguistics</t>
         </is>
       </c>
       <c r="C16" s="14" t="inlineStr">
         <is>
-          <t>De Anza PHIL 7 (Deductive Logic, or 7H honors) -- real equivalent, unlike EVC</t>
+          <t>De Anza LING 1 (Introduction to Linguistics) -- real equivalent, unlike EVC</t>
         </is>
       </c>
       <c r="D16" s="13" t="inlineStr"/>
@@ -2352,19 +2384,15 @@
       </c>
       <c r="B17" s="13" t="inlineStr">
         <is>
-          <t>multivar_calc</t>
+          <t>logic</t>
         </is>
       </c>
       <c r="C17" s="14" t="inlineStr">
         <is>
-          <t>De Anza MATH 1D (Calculus IV) -- satisfies UCI's MATH 2D/2E multivariable pair</t>
-        </is>
-      </c>
-      <c r="D17" s="13" t="inlineStr">
-        <is>
-          <t>calc3</t>
-        </is>
-      </c>
+          <t>De Anza PHIL 7 (Deductive Logic, or 7H honors) -- real equivalent, unlike EVC</t>
+        </is>
+      </c>
+      <c r="D17" s="13" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="13" t="inlineStr">
@@ -2374,17 +2402,17 @@
       </c>
       <c r="B18" s="13" t="inlineStr">
         <is>
-          <t>linear_algebra</t>
+          <t>multivar_calc</t>
         </is>
       </c>
       <c r="C18" s="14" t="inlineStr">
         <is>
-          <t>De Anza MATH 2B (or 2BH)</t>
+          <t>De Anza MATH 1D (Calculus IV) -- satisfies UCI's MATH 2D/2E multivariable pair</t>
         </is>
       </c>
       <c r="D18" s="13" t="inlineStr">
         <is>
-          <t>linalg</t>
+          <t>calc3</t>
         </is>
       </c>
     </row>
@@ -2396,17 +2424,17 @@
       </c>
       <c r="B19" s="13" t="inlineStr">
         <is>
-          <t>diffeq</t>
+          <t>linear_algebra</t>
         </is>
       </c>
       <c r="C19" s="14" t="inlineStr">
         <is>
-          <t>De Anza MATH 2A (or 2AH) -- note De Anza's OWN numbering: their 'MATH 2A' means Diff Eq, not Calc I</t>
+          <t>De Anza MATH 2B (or 2BH)</t>
         </is>
       </c>
       <c r="D19" s="13" t="inlineStr">
         <is>
-          <t>diffeq</t>
+          <t>linalg</t>
         </is>
       </c>
     </row>
@@ -2418,17 +2446,17 @@
       </c>
       <c r="B20" s="13" t="inlineStr">
         <is>
-          <t>physics_3course</t>
+          <t>diffeq</t>
         </is>
       </c>
       <c r="C20" s="14" t="inlineStr">
         <is>
-          <t>De Anza PHYS 2A/2B/2C (5 units, DEPRECATED next fall) OR PHYS 4A/4B/4C (6 units, use this one going forward)</t>
+          <t>De Anza MATH 2A (or 2AH) -- note De Anza's OWN numbering: their 'MATH 2A' means Diff Eq, not Calc I</t>
         </is>
       </c>
       <c r="D20" s="13" t="inlineStr">
         <is>
-          <t>physics1</t>
+          <t>diffeq</t>
         </is>
       </c>
     </row>
@@ -2440,17 +2468,17 @@
       </c>
       <c r="B21" s="13" t="inlineStr">
         <is>
-          <t>physics_3course</t>
+          <t>physics_calc_based</t>
         </is>
       </c>
       <c r="C21" s="14" t="inlineStr">
         <is>
-          <t>De Anza PHYS 2A/2B/2C (5 units, DEPRECATED next fall) OR PHYS 4A/4B/4C (6 units, use this one going forward)</t>
+          <t>De Anza PHYS 2A/2B/2C (5 units, DEPRECATED next fall) OR PHYS 4A/4B/4C (6 units, use this one going forward). This satisfies UCI's CALCULUS-BASED 'Classical Physics' sequence (PHYSICS 7C/7D/7E) specifically.</t>
         </is>
       </c>
       <c r="D21" s="13" t="inlineStr">
         <is>
-          <t>physics2</t>
+          <t>physics1</t>
         </is>
       </c>
     </row>
@@ -2462,17 +2490,17 @@
       </c>
       <c r="B22" s="13" t="inlineStr">
         <is>
-          <t>physics_3course</t>
+          <t>physics_calc_based</t>
         </is>
       </c>
       <c r="C22" s="14" t="inlineStr">
         <is>
-          <t>De Anza PHYS 2A/2B/2C (5 units, DEPRECATED next fall) OR PHYS 4A/4B/4C (6 units, use this one going forward)</t>
+          <t>De Anza PHYS 2A/2B/2C (5 units, DEPRECATED next fall) OR PHYS 4A/4B/4C (6 units, use this one going forward). This satisfies UCI's CALCULUS-BASED 'Classical Physics' sequence (PHYSICS 7C/7D/7E) specifically.</t>
         </is>
       </c>
       <c r="D22" s="13" t="inlineStr">
         <is>
-          <t>physics3</t>
+          <t>physics2</t>
         </is>
       </c>
     </row>
@@ -2484,68 +2512,64 @@
       </c>
       <c r="B23" s="13" t="inlineStr">
         <is>
-          <t>statistics</t>
+          <t>physics_calc_based</t>
         </is>
       </c>
       <c r="C23" s="14" t="inlineStr">
         <is>
-          <t>De Anza STAT C1000 (or Honors), or PSYC 15 / POLI 20 (same as SOC 15)</t>
+          <t>De Anza PHYS 2A/2B/2C (5 units, DEPRECATED next fall) OR PHYS 4A/4B/4C (6 units, use this one going forward). This satisfies UCI's CALCULUS-BASED 'Classical Physics' sequence (PHYSICS 7C/7D/7E) specifically.</t>
         </is>
       </c>
       <c r="D23" s="13" t="inlineStr">
         <is>
-          <t>stats_gen</t>
+          <t>physics3</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="13" t="inlineStr">
         <is>
-          <t>ucsd_cogsci_electives_evc</t>
+          <t>uci_cogsci_electives_deanza</t>
         </is>
       </c>
       <c r="B24" s="13" t="inlineStr">
         <is>
-          <t>neuro</t>
+          <t>physics_algebra_based</t>
         </is>
       </c>
       <c r="C24" s="14" t="inlineStr">
         <is>
-          <t>EVC PSYCH 030 (Intro Biological Psychology) -- likely satisfies a neuro-focused option</t>
-        </is>
-      </c>
-      <c r="D24" s="13" t="inlineStr">
-        <is>
-          <t>neuro_intro</t>
-        </is>
-      </c>
+          <t>UCI ALSO separately accepts an ALGEBRA-based 'Basic Physics' sequence (PHYSICS 3A/3B/3C) as an alternative option -- this is NOT the same course sequence as physics1/2/3 above and is NOT interchangeable with it (confirmed: user verified these are non-equivalent). No De Anza course has been confirmed against this specific algebra-based track -- do not assume the calc-based mapping above covers it.</t>
+        </is>
+      </c>
+      <c r="D24" s="13" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="13" t="inlineStr">
         <is>
-          <t>ucsd_cogsci_electives_evc</t>
+          <t>uci_cogsci_electives_deanza</t>
         </is>
       </c>
       <c r="B25" s="13" t="inlineStr">
         <is>
-          <t>programming</t>
+          <t>statistics</t>
         </is>
       </c>
       <c r="C25" s="14" t="inlineStr">
         <is>
-          <t>EVC COMSC 075, or CIT 044 (Java) + COMSC 076 combo -- ambiguous exact UCSD target course</t>
+          <t>De Anza STAT C1000 (or Honors), or PSYC 15 / POLI 20 (same as SOC 15)</t>
         </is>
       </c>
       <c r="D25" s="13" t="inlineStr">
         <is>
-          <t>prog1</t>
+          <t>stats_gen</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="13" t="inlineStr">
         <is>
-          <t>ucsd_cogsci_electives_deanza</t>
+          <t>ucsd_cogsci_electives_evc</t>
         </is>
       </c>
       <c r="B26" s="13" t="inlineStr">
@@ -2555,7 +2579,7 @@
       </c>
       <c r="C26" s="14" t="inlineStr">
         <is>
-          <t>De Anza PSYC 24 (Introduction to Psychobiology) -- likely satisfies COGS 17 Neurobiology of Cognition</t>
+          <t>EVC PSYCH 030 (Intro Biological Psychology) -- likely satisfies a neuro-focused option</t>
         </is>
       </c>
       <c r="D26" s="13" t="inlineStr">
@@ -2567,36 +2591,68 @@
     <row r="27">
       <c r="A27" s="13" t="inlineStr">
         <is>
+          <t>ucsd_cogsci_electives_evc</t>
+        </is>
+      </c>
+      <c r="B27" s="13" t="inlineStr">
+        <is>
+          <t>programming</t>
+        </is>
+      </c>
+      <c r="C27" s="14" t="inlineStr">
+        <is>
+          <t>EVC COMSC 075, or CIT 044 (Java) + COMSC 076 combo -- ambiguous exact UCSD target course</t>
+        </is>
+      </c>
+      <c r="D27" s="13" t="inlineStr">
+        <is>
+          <t>prog1</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="13" t="inlineStr">
+        <is>
           <t>ucsd_cogsci_electives_deanza</t>
         </is>
       </c>
-      <c r="B27" s="13" t="inlineStr">
+      <c r="B28" s="13" t="inlineStr">
+        <is>
+          <t>neuro</t>
+        </is>
+      </c>
+      <c r="C28" s="14" t="inlineStr">
+        <is>
+          <t>De Anza PSYC 24 (Introduction to Psychobiology) -- likely satisfies COGS 17 Neurobiology of Cognition</t>
+        </is>
+      </c>
+      <c r="D28" s="13" t="inlineStr">
+        <is>
+          <t>neuro_intro</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="13" t="inlineStr">
+        <is>
+          <t>ucsd_cogsci_electives_deanza</t>
+        </is>
+      </c>
+      <c r="B29" s="13" t="inlineStr">
         <is>
           <t>programming</t>
         </is>
       </c>
-      <c r="C27" s="14" t="inlineStr">
+      <c r="C29" s="14" t="inlineStr">
         <is>
           <t>De Anza: mostly 'No Course Articulated' for the COGS18/CSE6R/CSE8A/CSE11-style intro Python options; CIS 40 Python + CIS 41A, or CIS 35A/36B Java, may partially apply -- needs your visual check of the actual table</t>
         </is>
       </c>
-      <c r="D27" s="13" t="inlineStr">
+      <c r="D29" s="13" t="inlineStr">
         <is>
           <t>prog1</t>
         </is>
       </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="15" t="n"/>
-      <c r="B28" s="15" t="n"/>
-      <c r="C28" s="15" t="n"/>
-      <c r="D28" s="15" t="n"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="15" t="n"/>
-      <c r="B29" s="15" t="n"/>
-      <c r="C29" s="15" t="n"/>
-      <c r="D29" s="15" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="15" t="n"/>
@@ -2634,9 +2690,21 @@
       <c r="C35" s="15" t="n"/>
       <c r="D35" s="15" t="n"/>
     </row>
+    <row r="36">
+      <c r="A36" s="15" t="n"/>
+      <c r="B36" s="15" t="n"/>
+      <c r="C36" s="15" t="n"/>
+      <c r="D36" s="15" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="15" t="n"/>
+      <c r="B37" s="15" t="n"/>
+      <c r="C37" s="15" t="n"/>
+      <c r="D37" s="15" t="n"/>
+    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="D28 D29 D30 D31 D32 D33 D34 D35" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D30 D31 D32 D33 D34 D35 D36 D37" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"calc1,calc2,calc3,linalg,diffeq,discrete,prog1,prog2,comporg,digital_logic,physics1,physics2,physics3,circuits,stats_gen,linguistics,psych_intro,neuro_intro,cogsci_research,"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2645,6 +2713,246 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="70" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>school_key</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>AP Exam</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>Minimum Score</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>slot_id</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="13" t="inlineStr">
+        <is>
+          <t>ucsd</t>
+        </is>
+      </c>
+      <c r="B2" s="13" t="inlineStr">
+        <is>
+          <t>Calculus AB</t>
+        </is>
+      </c>
+      <c r="C2" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="D2" s="13" t="inlineStr">
+        <is>
+          <t>calc1</t>
+        </is>
+      </c>
+      <c r="E2" s="14" t="inlineStr">
+        <is>
+          <t>Exempts MATH 20A. AB score of 3 only exempts MATH 10A, a different sequence -- not counted as satisfying calc1 here.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="13" t="inlineStr">
+        <is>
+          <t>ucsd</t>
+        </is>
+      </c>
+      <c r="B3" s="13" t="inlineStr">
+        <is>
+          <t>Calculus BC</t>
+        </is>
+      </c>
+      <c r="C3" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="D3" s="13" t="inlineStr">
+        <is>
+          <t>calc1</t>
+        </is>
+      </c>
+      <c r="E3" s="14" t="inlineStr">
+        <is>
+          <t>Exempts MATH 20A (per official UC chart: 'exempt Mathematics 20A or 10A,10B').</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="13" t="inlineStr">
+        <is>
+          <t>ucsd</t>
+        </is>
+      </c>
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>Calculus BC</t>
+        </is>
+      </c>
+      <c r="C4" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="D4" s="13" t="inlineStr">
+        <is>
+          <t>calc2</t>
+        </is>
+      </c>
+      <c r="E4" s="14" t="inlineStr">
+        <is>
+          <t>Score of 4 or 5 exempts MATH 20A AND 20B. A BC score of 3 alone is NOT enough for calc2 -- only counted here at 4+.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="13" t="inlineStr">
+        <is>
+          <t>uci</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>Calculus AB</t>
+        </is>
+      </c>
+      <c r="C5" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="D5" s="13" t="inlineStr">
+        <is>
+          <t>calc1</t>
+        </is>
+      </c>
+      <c r="E5" s="14" t="inlineStr">
+        <is>
+          <t>Any passing AB score (3, 4, or 5) exempts MATH 2A per UCI's official AP credit chart.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="13" t="inlineStr">
+        <is>
+          <t>uci</t>
+        </is>
+      </c>
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>Calculus BC</t>
+        </is>
+      </c>
+      <c r="C6" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="D6" s="13" t="inlineStr">
+        <is>
+          <t>calc1</t>
+        </is>
+      </c>
+      <c r="E6" s="14" t="inlineStr">
+        <is>
+          <t>Exempts MATH 2A (places into MATH 2B).</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="13" t="inlineStr">
+        <is>
+          <t>uci</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>Calculus BC</t>
+        </is>
+      </c>
+      <c r="C7" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="D7" s="13" t="inlineStr">
+        <is>
+          <t>calc2</t>
+        </is>
+      </c>
+      <c r="E7" s="14" t="inlineStr">
+        <is>
+          <t>Score of 4 or 5 exempts MATH 2A AND 2B. A BC score of 3 alone only exempts 2A, not 2B -- only counted here at 4+.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="15" t="n"/>
+      <c r="B8" s="15" t="n"/>
+      <c r="C8" s="15" t="n"/>
+      <c r="D8" s="15" t="n"/>
+      <c r="E8" s="15" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="15" t="n"/>
+      <c r="B9" s="15" t="n"/>
+      <c r="C9" s="15" t="n"/>
+      <c r="D9" s="15" t="n"/>
+      <c r="E9" s="15" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="15" t="n"/>
+      <c r="B10" s="15" t="n"/>
+      <c r="C10" s="15" t="n"/>
+      <c r="D10" s="15" t="n"/>
+      <c r="E10" s="15" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="15" t="n"/>
+      <c r="B11" s="15" t="n"/>
+      <c r="C11" s="15" t="n"/>
+      <c r="D11" s="15" t="n"/>
+      <c r="E11" s="15" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="15" t="n"/>
+      <c r="B12" s="15" t="n"/>
+      <c r="C12" s="15" t="n"/>
+      <c r="D12" s="15" t="n"/>
+      <c r="E12" s="15" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="15" t="n"/>
+      <c r="B13" s="15" t="n"/>
+      <c r="C13" s="15" t="n"/>
+      <c r="D13" s="15" t="n"/>
+      <c r="E13" s="15" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>